<commit_message>
checkup run 2026-10-26: Check list (14 tickers); keep previous Friday-data run as 2026-10-25
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CiCmZq9JUHjQe2nY3AjisA
</commit_message>
<xml_diff>
--- a/checkup_data/Summary of 2026-10-26.xlsx
+++ b/checkup_data/Summary of 2026-10-26.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -673,11 +673,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>CLMT</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -695,40 +695,40 @@
         </is>
       </c>
       <c r="F2" s="7" t="n">
-        <v>325.43</v>
+        <v>52.17</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>3.653331634603152</v>
+        <v>5.810769698813512</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>253.284</v>
+        <v>42.00223333333334</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>0.6773627489310247</v>
+        <v>1.003068839329482</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>16.21356633467821</v>
+        <v>2.738227181169453</v>
       </c>
       <c r="K2" s="9" t="n">
-        <v>4.982197810490185</v>
+        <v>5.248662413589138</v>
       </c>
       <c r="L2" s="9" t="n">
-        <v>19.71695901991876</v>
+        <v>23.27683186073206</v>
       </c>
       <c r="M2" s="9" t="n">
-        <v>18.24838238943739</v>
+        <v>17.90610731497174</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>25.92464724494783</v>
+        <v>26.16862464384636</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>47.54372353463108</v>
+        <v>43.95566111899034</v>
       </c>
       <c r="P2" s="7" t="n">
-        <v>330.4849607379319</v>
+        <v>54.35479061790618</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>323.9212401084171</v>
+        <v>52.52953709670135</v>
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="S2" s="10" t="n">
-        <v>0.9875898105813196</v>
+        <v>0.7324380165289255</v>
       </c>
       <c r="T2" s="11" t="inlineStr">
         <is>
@@ -744,46 +744,46 @@
         </is>
       </c>
       <c r="U2" s="7" t="n">
-        <v>330.4849607379319</v>
+        <v>52.80976854835068</v>
       </c>
       <c r="V2" s="6" t="inlineStr">
         <is>
-          <t>EMA20</t>
+          <t>EMA50+גבוה אחרון</t>
         </is>
       </c>
       <c r="W2" s="9" t="n">
-        <v>0.3117735255518788</v>
+        <v>0.2336433414839737</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>342.67</v>
+        <v>54.12156197561976</v>
       </c>
       <c r="Y2" s="7" t="n">
-        <v>324.4937467028057</v>
+        <v>50</v>
       </c>
       <c r="Z2" s="6" t="inlineStr">
         <is>
-          <t>EMA50+גבוה קודם+גבוה אחרון</t>
+          <t>גבוה קודם</t>
         </is>
       </c>
       <c r="AA2" s="9" t="n">
-        <v>0.05774505607639222</v>
+        <v>0.7924835510080757</v>
       </c>
       <c r="AB2" s="7" t="n">
-        <v>308.58</v>
+        <v>48.18291666666666</v>
       </c>
       <c r="AC2" s="12" t="n">
-        <v>4630087.8</v>
+        <v>1688097.5</v>
       </c>
       <c r="AD2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>VIR</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -801,146 +801,146 @@
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>10.57</v>
+        <v>67.16</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>1.342281879194629</v>
+        <v>-0.6729276048214161</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>9.842666666666668</v>
+        <v>56.66706666666666</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1.109704057425613</v>
+        <v>0.7387119870023774</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.6067992128633843</v>
+        <v>5.448813982412269</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>5.740768333617638</v>
+        <v>8.113183416337506</v>
       </c>
       <c r="L3" s="9" t="n">
-        <v>15.21170428484271</v>
+        <v>18.65957120135771</v>
       </c>
       <c r="M3" s="9" t="n">
-        <v>18.7013695901973</v>
+        <v>14.85513641542361</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>22.62316128099064</v>
+        <v>18.18030444301736</v>
       </c>
       <c r="O3" s="9" t="n">
-        <v>47.83275106418854</v>
+        <v>46.67639836355405</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>10.72829893934329</v>
+        <v>69.23546332260577</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>10.58014424038961</v>
-      </c>
-      <c r="R3" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>67.53855284911239</v>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S3" s="10" t="n">
-        <v>0.3750000000000012</v>
+        <v>0.112923462986199</v>
       </c>
       <c r="T3" s="11" t="inlineStr">
         <is>
-          <t>בולעני עולה</t>
+          <t>פטיש (Hammer)</t>
         </is>
       </c>
       <c r="U3" s="7" t="n">
-        <v>10.66211079493322</v>
+        <v>68.23350404292954</v>
       </c>
       <c r="V3" s="6" t="inlineStr">
         <is>
-          <t>EMA50+גבוה אחרון+EMA20+גבוה קודם</t>
+          <t>EMA50+גבוה אחרון+גבוה קודם+EMA20</t>
         </is>
       </c>
       <c r="W3" s="9" t="n">
-        <v>0.1517978154562325</v>
+        <v>0.1970160931157878</v>
       </c>
       <c r="X3" s="7" t="n">
-        <v>11.11666666666667</v>
+        <v>76.23666666666666</v>
       </c>
       <c r="Y3" s="7" t="n">
-        <v>10.10333333333333</v>
+        <v>62.89840833333333</v>
       </c>
       <c r="Z3" s="6" t="inlineStr">
         <is>
-          <t>שפל חודש+נמוך אחרון+נמוך קודם+S1 M</t>
+          <t>שפל חודש+נמוך קודם+S1 M+נמוך אחרון</t>
         </is>
       </c>
       <c r="AA3" s="9" t="n">
-        <v>0.7690627422941843</v>
+        <v>0.7821136270062203</v>
       </c>
       <c r="AB3" s="7" t="n">
-        <v>9.406666666666668</v>
+        <v>44.86666666666666</v>
       </c>
       <c r="AC3" s="12" t="n">
-        <v>1526120.4</v>
+        <v>5098532.4</v>
       </c>
       <c r="AD3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>WTTR</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>מעורבת</t>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>יורדת ▼</t>
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>67.61499999999999</v>
+        <v>18.75</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>5.963015201379074</v>
+        <v>3.362734288864377</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>56.54693333333333</v>
+        <v>18.61993333333334</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>0.919500282166053</v>
+        <v>2.699863553189905</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>5.561415057982444</v>
+        <v>0.859116309216243</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>8.225120251397538</v>
+        <v>4.581953649153296</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>19.32065692470258</v>
+        <v>19.14321242269031</v>
       </c>
       <c r="M4" s="9" t="n">
-        <v>15.67393354084081</v>
+        <v>18.19556797665278</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>19.18238080239002</v>
+        <v>27.7997887498628</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>47.26912628466076</v>
+        <v>46.21428181387302</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>69.45393314603795</v>
+        <v>18.98472154900012</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>67.55400398581085</v>
+        <v>19.38759584109881</v>
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
@@ -948,54 +948,58 @@
         </is>
       </c>
       <c r="S4" s="10" t="n">
-        <v>0.6712696586114304</v>
+        <v>0.5286343612334824</v>
       </c>
       <c r="T4" s="11" t="inlineStr">
         <is>
-          <t>נר 2/3 ירוק אחרי אדום ▲</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U4" s="7" t="n">
-        <v>68.3607342829622</v>
+        <v>18.95324051633337</v>
       </c>
       <c r="V4" s="6" t="inlineStr">
         <is>
-          <t>EMA50+גבוה אחרון+גבוה קודם+EMA20</t>
+          <t>S1 M+EMA20+גבוה אחרון</t>
         </is>
       </c>
       <c r="W4" s="9" t="n">
-        <v>0.1340907440259888</v>
+        <v>0.236569267924603</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>76.23666666666666</v>
+        <v>19.38759584109881</v>
       </c>
       <c r="Y4" s="7" t="n">
-        <v>62.26840833333333</v>
+        <v>18.22</v>
       </c>
       <c r="Z4" s="6" t="inlineStr">
         <is>
-          <t>נמוך קודם+שפל חודש+נמוך אחרון+S1 M</t>
+          <t>גבוה קודם</t>
         </is>
       </c>
       <c r="AA4" s="9" t="n">
-        <v>0.96137253035854</v>
+        <v>0.6169129771072684</v>
       </c>
       <c r="AB4" s="7" t="n">
-        <v>44.86666666666666</v>
+        <v>17.885</v>
       </c>
       <c r="AC4" s="12" t="n">
-        <v>5101783.1</v>
-      </c>
-      <c r="AD4" s="11" t="inlineStr"/>
+        <v>1753503.8</v>
+      </c>
+      <c r="AD4" s="11" t="inlineStr">
+        <is>
+          <t>RVOL של טריידינגוויו (3.48) שונה מהחישוב לפי הנר האחרון (2.70); מגמת ירידה — לונג נגד המגמה</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>AMLX</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1013,70 +1017,70 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>70.84</v>
+        <v>27.09</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>2.355150989741372</v>
+        <v>-0.4044117647058809</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>66.80339999999997</v>
+        <v>21.56186666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>1.164501263431026</v>
+        <v>1.078087963167545</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2.340541487363697</v>
+        <v>1.458867229693779</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>3.303982901416851</v>
+        <v>5.385261091523732</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>20.07946547336601</v>
+        <v>20.76889162677006</v>
       </c>
       <c r="M5" s="9" t="n">
-        <v>11.68813270811146</v>
+        <v>18.89089965614095</v>
       </c>
       <c r="N5" s="9" t="n">
-        <v>29.11442671257992</v>
+        <v>30.20164664061447</v>
       </c>
       <c r="O5" s="9" t="n">
-        <v>42.45490554799343</v>
+        <v>42.234911597101</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>72.64964269869979</v>
+        <v>28.26155793379875</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>72.61493383777177</v>
-      </c>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>28.23907157622864</v>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S5" s="10" t="n">
-        <v>0.7326371622741595</v>
+        <v>0.09142857142857151</v>
       </c>
       <c r="T5" s="11" t="inlineStr">
         <is>
-          <t>נר 2/3 ירוק אחרי אדום ▲</t>
+          <t>דוג'י</t>
         </is>
       </c>
       <c r="U5" s="7" t="n">
-        <v>71.34333333333333</v>
+        <v>28.23515737750685</v>
       </c>
       <c r="V5" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון+S1 M</t>
+          <t>גבוה אחרון+EMA50+EMA20+גבוה קודם</t>
         </is>
       </c>
       <c r="W5" s="9" t="n">
-        <v>0.2150499514965945</v>
+        <v>0.784963397763908</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>72.56152551215719</v>
+        <v>30.14</v>
       </c>
       <c r="Y5" s="7" t="n">
-        <v>68.93000000000001</v>
+        <v>27.06</v>
       </c>
       <c r="Z5" s="6" t="inlineStr">
         <is>
@@ -1084,24 +1088,24 @@
         </is>
       </c>
       <c r="AA5" s="9" t="n">
-        <v>0.8160504781956899</v>
+        <v>0.02056390012016257</v>
       </c>
       <c r="AB5" s="7" t="n">
-        <v>68.00677777777777</v>
+        <v>26.66833333333334</v>
       </c>
       <c r="AC5" s="12" t="n">
-        <v>1423029.8</v>
+        <v>1271791.4</v>
       </c>
       <c r="AD5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1119,40 +1123,40 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>57.59</v>
+        <v>58.72</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.4885709300296748</v>
+        <v>3.580878461809855</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>52.68803333333337</v>
+        <v>46.12726666666669</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0.5868987523519467</v>
+        <v>0.4802353679315499</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>3.063586729077776</v>
+        <v>3.666865023678024</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>5.319650510640347</v>
+        <v>6.244661143865844</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>16.92458113323067</v>
+        <v>24.08972123564409</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>19.26100219266309</v>
+        <v>22.95446697451931</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>15.57085145749081</v>
+        <v>29.62901990396104</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>47.78096656965494</v>
+        <v>46.11067788532968</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>58.12922757065419</v>
+        <v>60.81821560140921</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>58.36652456849496</v>
+        <v>59.03484054972102</v>
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
@@ -1160,105 +1164,105 @@
         </is>
       </c>
       <c r="S6" s="10" t="n">
-        <v>0.2684563758389276</v>
+        <v>0.5837257267385287</v>
       </c>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>פטיש (Hammer)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U6" s="7" t="n">
-        <v>58.09141737971638</v>
+        <v>58.83536847076359</v>
       </c>
       <c r="V6" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון+EMA20+EMA50</t>
+          <t>גבוה קודם+Pivot M+EMA50+גבוה אחרון</t>
         </is>
       </c>
       <c r="W6" s="9" t="n">
-        <v>0.1636700456224132</v>
+        <v>0.0314624263556536</v>
       </c>
       <c r="X6" s="7" t="n">
-        <v>60.87763333333334</v>
+        <v>60.81821560140921</v>
       </c>
       <c r="Y6" s="7" t="n">
-        <v>55.34657777777778</v>
+        <v>56.83</v>
       </c>
       <c r="Z6" s="6" t="inlineStr">
         <is>
-          <t>S1 M+נמוך אחרון+נמוך קודם</t>
+          <t>נמוך אחרון</t>
         </is>
       </c>
       <c r="AA6" s="9" t="n">
-        <v>0.7322861797673191</v>
+        <v>0.5154266622293746</v>
       </c>
       <c r="AB6" s="7" t="n">
-        <v>54.265</v>
+        <v>54.275</v>
       </c>
       <c r="AC6" s="12" t="n">
-        <v>2078278.4</v>
+        <v>20321375</v>
       </c>
       <c r="AD6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>ERO</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>מעורבת</t>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>יורדת ▼</t>
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>88.08</v>
+        <v>31.21</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>-0.6317689530685899</v>
+        <v>4.207011686143569</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>86.63240000000012</v>
+        <v>30.58766666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1.318052763748952</v>
+        <v>1.130159354879502</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>3.799610351348735</v>
+        <v>1.802717689540381</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>4.313817383456784</v>
+        <v>5.776090001731436</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>26.19765148799778</v>
+        <v>19.73605464145724</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>12.51596406145854</v>
+        <v>18.20643033254227</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>32.95538646473919</v>
+        <v>32.72914011618118</v>
       </c>
       <c r="O7" s="9" t="n">
-        <v>36.99531564857084</v>
+        <v>37.55055083251817</v>
       </c>
       <c r="P7" s="7" t="n">
-        <v>94.92597437113275</v>
+        <v>34.04247130809856</v>
       </c>
       <c r="Q7" s="7" t="n">
-        <v>94.68855606748457</v>
+        <v>34.27083780289848</v>
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
@@ -1266,105 +1270,109 @@
         </is>
       </c>
       <c r="S7" s="10" t="n">
-        <v>0.3567839195979877</v>
+        <v>0.8187919463087253</v>
       </c>
       <c r="T7" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>נר 2/3 ירוק אחרי אדום ▲</t>
         </is>
       </c>
       <c r="U7" s="7" t="n">
-        <v>89.36001666666667</v>
+        <v>31.44</v>
       </c>
       <c r="V7" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון+S1 M</t>
+          <t>גבוה אחרון</t>
         </is>
       </c>
       <c r="W7" s="9" t="n">
-        <v>0.3368810347124949</v>
+        <v>0.1275851462125725</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>91.065</v>
+        <v>32.43333333333334</v>
       </c>
       <c r="Y7" s="7" t="n">
-        <v>87.15000000000001</v>
+        <v>30.51</v>
       </c>
       <c r="Z7" s="6" t="inlineStr">
         <is>
-          <t>נמוך אחרון</t>
+          <t>גבוה קודם</t>
         </is>
       </c>
       <c r="AA7" s="9" t="n">
-        <v>0.2447619397788706</v>
+        <v>0.3883026189078282</v>
       </c>
       <c r="AB7" s="7" t="n">
-        <v>85.66</v>
+        <v>29.76333333333334</v>
       </c>
       <c r="AC7" s="12" t="n">
-        <v>1307446.9</v>
-      </c>
-      <c r="AD7" s="11" t="inlineStr"/>
+        <v>1407613</v>
+      </c>
+      <c r="AD7" s="11" t="inlineStr">
+        <is>
+          <t>מגמת ירידה — לונג נגד המגמה</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NEO</t>
+          <t>EMBJ</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>מעורבת</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>יורדת ▼</t>
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.59</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1.220256253813301</v>
+        <v>0.3246753246753054</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>13.29726666666667</v>
+        <v>66.88579999999997</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.8683991046820257</v>
+        <v>1.697929963052083</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>0.8819597713131735</v>
+        <v>2.542645666837719</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>5.316213208638779</v>
+        <v>3.577663805878316</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>20.37085075611231</v>
+        <v>22.23986816424515</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>16.63868571119152</v>
+        <v>9.990585742729818</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>20.31381378133215</v>
+        <v>30.23329543422629</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>45.01923807875557</v>
+        <v>43.39852723451069</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>17.06556684258305</v>
+        <v>72.49920053691886</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>16.95738406837132</v>
+        <v>72.55434819707484</v>
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
@@ -1372,7 +1380,7 @@
         </is>
       </c>
       <c r="S8" s="10" t="n">
-        <v>0.333333333333335</v>
+        <v>0.4313346228239824</v>
       </c>
       <c r="T8" s="11" t="inlineStr">
         <is>
@@ -1380,46 +1388,50 @@
         </is>
       </c>
       <c r="U8" s="7" t="n">
-        <v>16.95053684885754</v>
+        <v>71.37222222222222</v>
       </c>
       <c r="V8" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון+S1 M+EMA50+EMA20+גבוה קודם</t>
+          <t>גבוה קודם+גבוה אחרון+S1 M</t>
         </is>
       </c>
       <c r="W8" s="9" t="n">
-        <v>0.4087905827277425</v>
+        <v>0.1188613207746322</v>
       </c>
       <c r="X8" s="7" t="n">
-        <v>18.42496666666667</v>
+        <v>72.52677436699685</v>
       </c>
       <c r="Y8" s="7" t="n">
-        <v>16.095</v>
+        <v>67.92841666666666</v>
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
-          <t>נמוך אחרון+נמוך קודם</t>
+          <t>S2 M+נמוך קודם</t>
         </is>
       </c>
       <c r="AA8" s="9" t="n">
-        <v>0.5612500888367984</v>
+        <v>1.235556874600033</v>
       </c>
       <c r="AB8" s="7" t="n">
-        <v>15.32503333333333</v>
+        <v>66.26000000000001</v>
       </c>
       <c r="AC8" s="12" t="n">
-        <v>1648397.6</v>
-      </c>
-      <c r="AD8" s="11" t="inlineStr"/>
+        <v>1652704.8</v>
+      </c>
+      <c r="AD8" s="11" t="inlineStr">
+        <is>
+          <t>מגמת ירידה — לונג נגד המגמה</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1437,95 +1449,95 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>646.15</v>
+        <v>148.53</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.3930890898356187</v>
+        <v>-2.769049489395126</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>611.1743333333322</v>
+        <v>139.8595000000001</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.6661213804757276</v>
+        <v>1.150219680754552</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>17.64830324033239</v>
+        <v>4.364807151022502</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>2.731301283035269</v>
+        <v>2.938670403973946</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>19.20403553852847</v>
+        <v>11.2997235023435</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>19.60166340378633</v>
+        <v>18.24551215515989</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>26.49216844269711</v>
+        <v>22.41673014807249</v>
       </c>
       <c r="O9" s="9" t="n">
-        <v>46.65416616891198</v>
+        <v>40.24967166054985</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>651.3929980082709</v>
+        <v>154.243733392566</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>650.8134270459847</v>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>153.66559738204</v>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S9" s="10" t="n">
-        <v>0.3351084062381088</v>
+        <v>0.5416036308623305</v>
       </c>
       <c r="T9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>נר אדום</t>
         </is>
       </c>
       <c r="U9" s="7" t="n">
-        <v>651.1032125271278</v>
+        <v>151.805</v>
       </c>
       <c r="V9" s="6" t="inlineStr">
         <is>
-          <t>EMA50+EMA20</t>
+          <t>S1 M+נמוך קודם</t>
         </is>
       </c>
       <c r="W9" s="9" t="n">
-        <v>0.2806622517573253</v>
+        <v>0.7503195185227834</v>
       </c>
       <c r="X9" s="7" t="n">
-        <v>682.2733333333333</v>
+        <v>153.9164435915353</v>
       </c>
       <c r="Y9" s="7" t="n">
-        <v>644.7588888888889</v>
+        <v>146.9966666666667</v>
       </c>
       <c r="Z9" s="6" t="inlineStr">
         <is>
-          <t>S1 M+גבוה קודם+גבוה אחרון</t>
+          <t>S2 M+נמוך אחרון+שפל חודש</t>
         </is>
       </c>
       <c r="AA9" s="9" t="n">
-        <v>0.07882407119636833</v>
+        <v>0.3512946346264421</v>
       </c>
       <c r="AB9" s="7" t="n">
-        <v>633.0549999999999</v>
+        <v>141.05</v>
       </c>
       <c r="AC9" s="12" t="n">
-        <v>1041777.1</v>
+        <v>3846946</v>
       </c>
       <c r="AD9" s="11" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CMBT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1543,40 +1555,40 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>18.46</v>
+        <v>216</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>2.101769911504436</v>
+        <v>2.389078498293506</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>16.0832</v>
+        <v>210.2894666666666</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.3504437331631503</v>
+        <v>0.8930652185841758</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.6874995578055426</v>
+        <v>6.113715040536869</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>3.724266293637826</v>
+        <v>2.83042362987818</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>27.09419719562686</v>
+        <v>18.89859889558345</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>25.46551224350165</v>
+        <v>21.20782923857999</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>29.42054113940606</v>
+        <v>29.76839794703326</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>46.36927873307313</v>
+        <v>44.11780126818738</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>18.81393371500638</v>
+        <v>221.0347886496322</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>18.52369569437863</v>
+        <v>220.7018764973952</v>
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
@@ -1584,7 +1596,7 @@
         </is>
       </c>
       <c r="S10" s="10" t="n">
-        <v>0.6166666666666705</v>
+        <v>0.5632295719844392</v>
       </c>
       <c r="T10" s="11" t="inlineStr">
         <is>
@@ -1592,46 +1604,46 @@
         </is>
       </c>
       <c r="U10" s="7" t="n">
-        <v>18.66254313646167</v>
+        <v>217.75</v>
       </c>
       <c r="V10" s="6" t="inlineStr">
         <is>
-          <t>EMA50+גבוה אחרון+EMA20</t>
+          <t>גבוה אחרון</t>
         </is>
       </c>
       <c r="W10" s="9" t="n">
-        <v>0.2946083879794378</v>
+        <v>0.2862416694917344</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>19.28666666666667</v>
+        <v>220.8683325735137</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>18.3</v>
+        <v>213.2488888888889</v>
       </c>
       <c r="Z10" s="6" t="inlineStr">
         <is>
-          <t>גבוה קודם</t>
+          <t>נמוך אחרון+S1 M+גבוה קודם</t>
         </is>
       </c>
       <c r="AA10" s="9" t="n">
-        <v>0.2327274224156748</v>
+        <v>0.4499900785152582</v>
       </c>
       <c r="AB10" s="7" t="n">
-        <v>18.05</v>
+        <v>210.18</v>
       </c>
       <c r="AC10" s="12" t="n">
-        <v>1576341.5</v>
+        <v>101251856.1</v>
       </c>
       <c r="AD10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AME</t>
+          <t>OMDA</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -1643,46 +1655,46 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>מעורבת</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>יורדת ▼</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>240.03</v>
+        <v>19.24</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.5066577338581402</v>
+        <v>1.530343007915569</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>236.2988666666668</v>
+        <v>18.90540000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.7613386575927481</v>
+        <v>0.7010713019760988</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>5.828673013840709</v>
+        <v>1.019226658471305</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>2.428310216989838</v>
+        <v>5.297435854840461</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>13.35884275198005</v>
+        <v>17.27876362095637</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>16.66460680411273</v>
+        <v>19.96882728697345</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>32.809791435964</v>
+        <v>28.02920486054555</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>40.91251199424946</v>
+        <v>46.00835292955423</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>246.2410807854998</v>
+        <v>19.59073947516242</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>244.491986940217</v>
+        <v>20.35860636916784</v>
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
@@ -1690,7 +1702,7 @@
         </is>
       </c>
       <c r="S11" s="10" t="n">
-        <v>0.61821086261981</v>
+        <v>0.3716814159291979</v>
       </c>
       <c r="T11" s="11" t="inlineStr">
         <is>
@@ -1698,50 +1710,54 @@
         </is>
       </c>
       <c r="U11" s="7" t="n">
-        <v>241.42</v>
+        <v>19.43857982505414</v>
       </c>
       <c r="V11" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון</t>
+          <t>גבוה קודם+גבוה אחרון+EMA20</t>
         </is>
       </c>
       <c r="W11" s="9" t="n">
-        <v>0.2384762357914582</v>
+        <v>0.1948338217055477</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>244.1656601367752</v>
+        <v>20.35860636916784</v>
       </c>
       <c r="Y11" s="7" t="n">
-        <v>234.3764166666667</v>
+        <v>18.785</v>
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
-          <t>S1 M+נמוך קודם+שפל חודש+נמוך אחרון</t>
+          <t>נמוך קודם+נמוך אחרון</t>
         </is>
       </c>
       <c r="AA11" s="9" t="n">
-        <v>0.9699606273860941</v>
+        <v>0.4464168948273329</v>
       </c>
       <c r="AB11" s="7" t="n">
-        <v>229.595</v>
+        <v>18.13333333333333</v>
       </c>
       <c r="AC11" s="12" t="n">
-        <v>1298784.7</v>
-      </c>
-      <c r="AD11" s="11" t="inlineStr"/>
+        <v>1241582.7</v>
+      </c>
+      <c r="AD11" s="11" t="inlineStr">
+        <is>
+          <t>מגמת ירידה — לונג נגד המגמה</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+        <v>28</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>❌</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1755,40 +1771,40 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>28.98</v>
+        <v>326.04</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>1.151832460732982</v>
+        <v>3.580392032277557</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>27.42786666666664</v>
+        <v>335.6003333333333</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.6224096188725966</v>
+        <v>1.007904757688431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>0.8737019951011257</v>
+        <v>13.7015376470564</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>3.014844703592566</v>
+        <v>4.202410025474298</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>13.93490353399982</v>
+        <v>30.96728854554108</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>21.92586489749913</v>
+        <v>19.03749647059424</v>
       </c>
       <c r="N12" s="9" t="n">
-        <v>21.56276145180697</v>
+        <v>40.74633182800274</v>
       </c>
       <c r="O12" s="9" t="n">
-        <v>46.25585577096323</v>
+        <v>41.0537879668951</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>29.23060320335364</v>
+        <v>344.1574979653222</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>29.42654641260913</v>
+        <v>343.717391630553</v>
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
@@ -1796,7 +1812,7 @@
         </is>
       </c>
       <c r="S12" s="10" t="n">
-        <v>0.3771428571428593</v>
+        <v>0.5729296771126292</v>
       </c>
       <c r="T12" s="11" t="inlineStr">
         <is>
@@ -1804,97 +1820,97 @@
         </is>
       </c>
       <c r="U12" s="7" t="n">
-        <v>29.36238320532092</v>
+        <v>328.3213166666667</v>
       </c>
       <c r="V12" s="6" t="inlineStr">
         <is>
-          <t>EMA20+EMA50+גבוה אחרון</t>
+          <t>S1 M+גבוה אחרון</t>
         </is>
       </c>
       <c r="W12" s="9" t="n">
-        <v>0.4376586152543525</v>
+        <v>0.1665007771705667</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>30.39333333333333</v>
+        <v>345.1090520875139</v>
       </c>
       <c r="Y12" s="7" t="n">
-        <v>28.95</v>
+        <v>316.795</v>
       </c>
       <c r="Z12" s="6" t="inlineStr">
         <is>
-          <t>גבוה קודם</t>
+          <t>נמוך אחרון+גבוה קודם</t>
         </is>
       </c>
       <c r="AA12" s="9" t="n">
-        <v>0.03433665044627582</v>
+        <v>0.6747417872465015</v>
       </c>
       <c r="AB12" s="7" t="n">
-        <v>28.555</v>
+        <v>305.01</v>
       </c>
       <c r="AC12" s="12" t="n">
-        <v>1409179.7</v>
+        <v>1391415.2</v>
       </c>
       <c r="AD12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>WTTR</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>מעורבת</t>
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>18.14</v>
+        <v>140.22</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>3.420752565564422</v>
+        <v>4.237288135593209</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>18.59113333333334</v>
+        <v>142.6786333333333</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1.538287450886114</v>
+        <v>0.9278572675040501</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.837894486848262</v>
+        <v>8.446142840658162</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>4.619043477664068</v>
+        <v>6.023493681827245</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>19.00954810602207</v>
+        <v>20.60113675654232</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>12.42579153261332</v>
+        <v>20.67370468651909</v>
       </c>
       <c r="N13" s="9" t="n">
-        <v>30.69649643858566</v>
+        <v>33.00697590472758</v>
       </c>
       <c r="O13" s="9" t="n">
-        <v>39.90052484189107</v>
+        <v>44.79087594112084</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>19.00942908047382</v>
+        <v>146.9614346258963</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>19.41362016114366</v>
+        <v>146.794703374472</v>
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
@@ -1902,15 +1918,15 @@
         </is>
       </c>
       <c r="S13" s="10" t="n">
-        <v>0.6705882352941197</v>
+        <v>0.5924479166666698</v>
       </c>
       <c r="T13" s="11" t="inlineStr">
         <is>
-          <t>נר 2/3 ירוק אחרי אדום ▲</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U13" s="7" t="n">
-        <v>18.22</v>
+        <v>142.2</v>
       </c>
       <c r="V13" s="6" t="inlineStr">
         <is>
@@ -1918,46 +1934,42 @@
         </is>
       </c>
       <c r="W13" s="9" t="n">
-        <v>0.09547741542126395</v>
+        <v>0.2344265349703344</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>18.84980969349127</v>
+        <v>146.4176015556783</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>17.85</v>
+        <v>134.5911111111111</v>
       </c>
       <c r="Z13" s="6" t="inlineStr">
         <is>
-          <t>S2 M</t>
+          <t>S1 M+נמוך אחרון+גבוה קודם</t>
         </is>
       </c>
       <c r="AA13" s="9" t="n">
-        <v>0.3461056309020882</v>
+        <v>0.666444908058205</v>
       </c>
       <c r="AB13" s="7" t="n">
-        <v>17.37</v>
+        <v>127.01</v>
       </c>
       <c r="AC13" s="12" t="n">
-        <v>1362267.5</v>
-      </c>
-      <c r="AD13" s="11" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
+        <v>2815381.3</v>
+      </c>
+      <c r="AD13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CLBK</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+        <v>23</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>❌</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1971,40 +1983,40 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>10.85</v>
+        <v>818.1</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>-0.09208103130754486</v>
+        <v>8.18995728473757</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>9.966889274933324</v>
+        <v>871.8491999999995</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>0.732176079083439</v>
+        <v>1.199889745734583</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>0.2425066235696663</v>
+        <v>69.91425892784027</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>2.235084088199689</v>
+        <v>8.545930684248901</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>22.24764470918985</v>
+        <v>22.57197175473508</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>16.77439734031707</v>
+        <v>21.80185674942494</v>
       </c>
       <c r="N14" s="9" t="n">
-        <v>21.8267523965496</v>
+        <v>33.80449398013079</v>
       </c>
       <c r="O14" s="9" t="n">
-        <v>45.67886883597718</v>
+        <v>41.72994078223007</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>10.91408966413119</v>
+        <v>893.1052737535183</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>10.9929487694882</v>
+        <v>905.7065765396655</v>
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
@@ -2012,7 +2024,7 @@
         </is>
       </c>
       <c r="S14" s="10" t="n">
-        <v>0.1599999999999966</v>
+        <v>0.6129986977625187</v>
       </c>
       <c r="T14" s="11" t="inlineStr">
         <is>
@@ -2020,35 +2032,35 @@
         </is>
       </c>
       <c r="U14" s="7" t="n">
-        <v>10.90302988804373</v>
+        <v>845.825</v>
       </c>
       <c r="V14" s="6" t="inlineStr">
         <is>
-          <t>גבוה קודם+EMA20+גבוה אחרון</t>
+          <t>גבוה אחרון+S1 M</t>
         </is>
       </c>
       <c r="W14" s="9" t="n">
-        <v>0.2186739779026993</v>
+        <v>0.3965571605159325</v>
       </c>
       <c r="X14" s="7" t="n">
-        <v>10.9929487694882</v>
+        <v>899.4059251465919</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>10.79</v>
+        <v>788.8952</v>
       </c>
       <c r="Z14" s="6" t="inlineStr">
         <is>
-          <t>נמוך אחרון</t>
+          <t>גבוה קודם</t>
         </is>
       </c>
       <c r="AA14" s="9" t="n">
-        <v>0.2474159225707249</v>
+        <v>0.4177230860752277</v>
       </c>
       <c r="AB14" s="7" t="n">
-        <v>10.55791666666667</v>
+        <v>756</v>
       </c>
       <c r="AC14" s="12" t="n">
-        <v>2930292.4</v>
+        <v>5010237</v>
       </c>
       <c r="AD14" s="11" t="inlineStr">
         <is>
@@ -2059,11 +2071,11 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>MXL</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -2081,40 +2093,40 @@
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>175.91</v>
+        <v>66.47</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>1.782098015390843</v>
+        <v>4.743145288370632</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>177.169733333334</v>
+        <v>72.51186666666665</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.7131512653603199</v>
+        <v>0.9095604970377704</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>6.792276354965082</v>
+        <v>7.859584470801532</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>3.861222417693754</v>
+        <v>11.82425826809317</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>9.24863127661922</v>
+        <v>23.85196024232869</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>16.72239074144698</v>
+        <v>19.32177951301562</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>17.7547338989276</v>
+        <v>33.54277802783173</v>
       </c>
       <c r="O15" s="9" t="n">
-        <v>47.94910579439705</v>
+        <v>38.79191830078187</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>177.4733515110907</v>
+        <v>78.91856743114118</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>177.7213468603753</v>
+        <v>79.43669052237664</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -2122,43 +2134,43 @@
         </is>
       </c>
       <c r="S15" s="10" t="n">
-        <v>0.6981818181818188</v>
+        <v>0.3511197874301824</v>
       </c>
       <c r="T15" s="11" t="inlineStr">
         <is>
-          <t>נר 2/3 ירוק אחרי אדום ▲, בולעני עולה</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U15" s="7" t="n">
-        <v>177.7174245928665</v>
+        <v>68.7988</v>
       </c>
       <c r="V15" s="6" t="inlineStr">
         <is>
-          <t>גבוה אחרון+EMA20+EMA50+גבוה קודם</t>
+          <t>גבוה אחרון</t>
         </is>
       </c>
       <c r="W15" s="9" t="n">
-        <v>0.2660999786242947</v>
+        <v>0.2963006515995249</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>184.0344</v>
+        <v>79.72508598450594</v>
       </c>
       <c r="Y15" s="7" t="n">
-        <v>171.7025</v>
+        <v>65.78999999999999</v>
       </c>
       <c r="Z15" s="6" t="inlineStr">
         <is>
-          <t>נמוך אחרון+נמוך קודם</t>
+          <t>S1 M+גבוה קודם</t>
         </is>
       </c>
       <c r="AA15" s="9" t="n">
-        <v>0.6194535940700311</v>
+        <v>0.08651856882844335</v>
       </c>
       <c r="AB15" s="7" t="n">
-        <v>168.84</v>
+        <v>61.4224</v>
       </c>
       <c r="AC15" s="12" t="n">
-        <v>10174291.7</v>
+        <v>3986473.7</v>
       </c>
       <c r="AD15" s="11" t="inlineStr">
         <is>
@@ -2166,448 +2178,8 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>CXW</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>30.04</v>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>2.420729628366858</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>27.72799999999999</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>0.7433824513027116</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>1.564140491380076</v>
-      </c>
-      <c r="K16" s="9" t="n">
-        <v>5.206859159054847</v>
-      </c>
-      <c r="L16" s="9" t="n">
-        <v>19.48017057173068</v>
-      </c>
-      <c r="M16" s="9" t="n">
-        <v>16.00106820814626</v>
-      </c>
-      <c r="N16" s="9" t="n">
-        <v>30.80350727636675</v>
-      </c>
-      <c r="O16" s="9" t="n">
-        <v>40.70273313475275</v>
-      </c>
-      <c r="P16" s="7" t="n">
-        <v>31.54250398220144</v>
-      </c>
-      <c r="Q16" s="7" t="n">
-        <v>31.97147835384928</v>
-      </c>
-      <c r="R16" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
-        </is>
-      </c>
-      <c r="S16" s="10" t="n">
-        <v>0.6320754716981122</v>
-      </c>
-      <c r="T16" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="V16" s="6" t="inlineStr">
-        <is>
-          <t>גבוה אחרון</t>
-        </is>
-      </c>
-      <c r="W16" s="9" t="n">
-        <v>0.2301583534113124</v>
-      </c>
-      <c r="X16" s="7" t="n">
-        <v>31.54250398220144</v>
-      </c>
-      <c r="Y16" s="7" t="n">
-        <v>29.55444444444445</v>
-      </c>
-      <c r="Z16" s="6" t="inlineStr">
-        <is>
-          <t>נמוך אחרון+גבוה קודם+S1 M</t>
-        </is>
-      </c>
-      <c r="AA16" s="9" t="n">
-        <v>0.3104296309899482</v>
-      </c>
-      <c r="AB16" s="7" t="n">
-        <v>28.43</v>
-      </c>
-      <c r="AC16" s="12" t="n">
-        <v>1638612.8</v>
-      </c>
-      <c r="AD16" s="11" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>MAN</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>47.53</v>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>1.995708154506448</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>42.70113333333333</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>0.7659428918626392</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>2.596679866473348</v>
-      </c>
-      <c r="K17" s="9" t="n">
-        <v>5.463243985847566</v>
-      </c>
-      <c r="L17" s="9" t="n">
-        <v>41.38397724188626</v>
-      </c>
-      <c r="M17" s="9" t="n">
-        <v>20.68840694345327</v>
-      </c>
-      <c r="N17" s="9" t="n">
-        <v>32.92007171825394</v>
-      </c>
-      <c r="O17" s="9" t="n">
-        <v>41.49401795381126</v>
-      </c>
-      <c r="P17" s="7" t="n">
-        <v>49.45300212098536</v>
-      </c>
-      <c r="Q17" s="7" t="n">
-        <v>51.86697073178766</v>
-      </c>
-      <c r="R17" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
-        </is>
-      </c>
-      <c r="S17" s="10" t="n">
-        <v>0.6367112810707466</v>
-      </c>
-      <c r="T17" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="n">
-        <v>48.48</v>
-      </c>
-      <c r="V17" s="6" t="inlineStr">
-        <is>
-          <t>גבוה אחרון</t>
-        </is>
-      </c>
-      <c r="W17" s="9" t="n">
-        <v>0.3658517987780402</v>
-      </c>
-      <c r="X17" s="7" t="n">
-        <v>49.49316772715935</v>
-      </c>
-      <c r="Y17" s="7" t="n">
-        <v>46.745</v>
-      </c>
-      <c r="Z17" s="6" t="inlineStr">
-        <is>
-          <t>גבוה קודם</t>
-        </is>
-      </c>
-      <c r="AA17" s="9" t="n">
-        <v>0.3023091179376465</v>
-      </c>
-      <c r="AB17" s="7" t="n">
-        <v>45.865</v>
-      </c>
-      <c r="AC17" s="12" t="n">
-        <v>1490463.6</v>
-      </c>
-      <c r="AD17" s="11" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>NTRS</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>167.92</v>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>1.266433482089013</v>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>171.5029</v>
-      </c>
-      <c r="I18" s="7" t="n">
-        <v>1.015681882806071</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>3.961835963448979</v>
-      </c>
-      <c r="K18" s="9" t="n">
-        <v>2.359359196908635</v>
-      </c>
-      <c r="L18" s="9" t="n">
-        <v>33.596926086235</v>
-      </c>
-      <c r="M18" s="9" t="n">
-        <v>19.72274234534433</v>
-      </c>
-      <c r="N18" s="9" t="n">
-        <v>25.65687296591571</v>
-      </c>
-      <c r="O18" s="9" t="n">
-        <v>43.98241747569945</v>
-      </c>
-      <c r="P18" s="7" t="n">
-        <v>168.839633094039</v>
-      </c>
-      <c r="Q18" s="7" t="n">
-        <v>173.6555897900118</v>
-      </c>
-      <c r="R18" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
-        </is>
-      </c>
-      <c r="S18" s="10" t="n">
-        <v>0.719290051377857</v>
-      </c>
-      <c r="T18" s="11" t="inlineStr">
-        <is>
-          <t>נר גוף מלא ירוק</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="n">
-        <v>168.8060665470195</v>
-      </c>
-      <c r="V18" s="6" t="inlineStr">
-        <is>
-          <t>גבוה אחרון+EMA20</t>
-        </is>
-      </c>
-      <c r="W18" s="9" t="n">
-        <v>0.2236504881055632</v>
-      </c>
-      <c r="X18" s="7" t="n">
-        <v>173.6555897900118</v>
-      </c>
-      <c r="Y18" s="7" t="n">
-        <v>167.585</v>
-      </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>גבוה קודם</t>
-        </is>
-      </c>
-      <c r="AA18" s="9" t="n">
-        <v>0.08455675678917939</v>
-      </c>
-      <c r="AB18" s="7" t="n">
-        <v>163.33</v>
-      </c>
-      <c r="AC18" s="12" t="n">
-        <v>1485510.4</v>
-      </c>
-      <c r="AD18" s="11" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>HTGC</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>16.41</v>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>-0.4851425106124796</v>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>16.12846666666668</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>0.8764241514147624</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>0.2987116680015121</v>
-      </c>
-      <c r="K19" s="9" t="n">
-        <v>1.820302669113419</v>
-      </c>
-      <c r="L19" s="9" t="n">
-        <v>26.40256412821574</v>
-      </c>
-      <c r="M19" s="9" t="n">
-        <v>17.24429278215446</v>
-      </c>
-      <c r="N19" s="9" t="n">
-        <v>23.61765731412448</v>
-      </c>
-      <c r="O19" s="9" t="n">
-        <v>44.08517042572382</v>
-      </c>
-      <c r="P19" s="7" t="n">
-        <v>16.56228394144973</v>
-      </c>
-      <c r="Q19" s="7" t="n">
-        <v>16.72134326087678</v>
-      </c>
-      <c r="R19" s="6" t="inlineStr">
-        <is>
-          <t>ניטרלי</t>
-        </is>
-      </c>
-      <c r="S19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="11" t="inlineStr">
-        <is>
-          <t>דוג'י</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="n">
-        <v>16.53042798048324</v>
-      </c>
-      <c r="V19" s="6" t="inlineStr">
-        <is>
-          <t>גבוה אחרון+גבוה קודם+EMA20</t>
-        </is>
-      </c>
-      <c r="W19" s="9" t="n">
-        <v>0.4031579391891475</v>
-      </c>
-      <c r="X19" s="7" t="n">
-        <v>16.72134326087678</v>
-      </c>
-      <c r="Y19" s="7" t="n">
-        <v>16.37650000000001</v>
-      </c>
-      <c r="Z19" s="6" t="inlineStr">
-        <is>
-          <t>S1 M</t>
-        </is>
-      </c>
-      <c r="AA19" s="9" t="n">
-        <v>0.1121482807287709</v>
-      </c>
-      <c r="AB19" s="7" t="n">
-        <v>16.23</v>
-      </c>
-      <c r="AC19" s="12" t="n">
-        <v>1017676.2</v>
-      </c>
-      <c r="AD19" s="11" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B19">
+  <conditionalFormatting sqref="B2:B15">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2644,7 +2216,7 @@
       </c>
       <c r="B1" s="14" t="inlineStr">
         <is>
-          <t>רשימת המעקב 'Check list' בטריידינגוויו, גרף יומי. נר אחרון: 2026-10-23</t>
+          <t>רשימת המעקב 'Check list' בטריידינגוויו, גרף יומי. נר אחרון: 2026-10-26</t>
         </is>
       </c>
     </row>

</xml_diff>